<commit_message>
Horizontal GridLine Change, Delta movment opimization
</commit_message>
<xml_diff>
--- a/cmd/big/specimen.xlsx
+++ b/cmd/big/specimen.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29426"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29628"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="Z:\go\src\github.com\tranners\fyne-xlsx\cmd\big\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E4C2FB5C-AA26-481F-B715-D9E6AE032502}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{13CCE0FF-8C25-410D-9C1D-2204A5A7F9AB}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="51840" windowHeight="20445" xr2:uid="{18453F22-C442-461A-B1D5-BC6CD41F0A82}"/>
   </bookViews>
@@ -224,7 +224,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="10">
+  <fills count="11">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -263,12 +263,6 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFF0000"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
         <fgColor theme="8" tint="0.39994506668294322"/>
         <bgColor indexed="64"/>
       </patternFill>
@@ -276,6 +270,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="1"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="7" tint="0.59996337778862885"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor theme="9" tint="0.59996337778862885"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1196,7 +1202,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="111">
+  <cellXfs count="115">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
@@ -1246,7 +1252,6 @@
       <alignment horizontal="right" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="22" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="7" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="23" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="top"/>
     </xf>
@@ -1339,69 +1344,80 @@
     <xf numFmtId="0" fontId="0" fillId="4" borderId="15" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="32" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="33" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="34" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="35" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="36" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="37" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="38" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="9" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="7" fillId="8" borderId="39" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="26" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="27" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="29" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="28" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="30" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="8" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="7" borderId="31" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="9" fillId="9" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="76" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="77" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="78" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="68" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="69" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="70" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="71" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="72" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="73" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="74" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="9" fillId="8" borderId="75" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1837,11 +1853,11 @@
         <f t="shared" si="0"/>
         <v>24</v>
       </c>
-      <c r="Y1" s="54">
+      <c r="Y1" s="53">
         <f>ROW()*COLUMN()</f>
         <v>25</v>
       </c>
-      <c r="Z1" s="55">
+      <c r="Z1" s="54">
         <f t="shared" ref="Z1:AT13" si="1">ROW()*COLUMN()</f>
         <v>26</v>
       </c>
@@ -2083,12 +2099,10 @@
       <c r="D2" s="20">
         <v>1</v>
       </c>
-      <c r="E2" s="20">
-        <v>1</v>
-      </c>
-      <c r="F2" s="20">
-        <v>1</v>
-      </c>
+      <c r="E2" s="113">
+        <v>1</v>
+      </c>
+      <c r="F2" s="113"/>
       <c r="G2" s="20">
         <v>1</v>
       </c>
@@ -2101,16 +2115,16 @@
       <c r="J2" s="20">
         <v>2</v>
       </c>
-      <c r="K2" s="39" t="s">
+      <c r="K2" s="38" t="s">
         <v>31</v>
       </c>
-      <c r="L2" s="40">
+      <c r="L2" s="39">
         <v>2</v>
       </c>
-      <c r="M2" s="40">
+      <c r="M2" s="39">
         <v>2</v>
       </c>
-      <c r="N2" s="34" t="s">
+      <c r="N2" s="33" t="s">
         <v>6</v>
       </c>
       <c r="O2" t="s">
@@ -2122,12 +2136,10 @@
       <c r="Q2" s="13" t="s">
         <v>3</v>
       </c>
-      <c r="R2">
+      <c r="R2" s="111">
         <v>44</v>
       </c>
-      <c r="S2">
-        <v>22</v>
-      </c>
+      <c r="S2" s="111"/>
       <c r="T2">
         <f t="shared" ref="T2:AI30" si="4">ROW()*COLUMN()</f>
         <v>40</v>
@@ -2148,11 +2160,11 @@
         <f t="shared" si="4"/>
         <v>48</v>
       </c>
-      <c r="Y2" s="54">
+      <c r="Y2" s="53">
         <f t="shared" si="4"/>
         <v>50</v>
       </c>
-      <c r="Z2" s="55">
+      <c r="Z2" s="54">
         <v>6</v>
       </c>
       <c r="AA2">
@@ -2393,12 +2405,8 @@
       <c r="D3" s="20">
         <v>1</v>
       </c>
-      <c r="E3" s="20">
-        <v>1</v>
-      </c>
-      <c r="F3" s="20">
-        <v>1</v>
-      </c>
+      <c r="E3" s="113"/>
+      <c r="F3" s="113"/>
       <c r="G3" s="20">
         <v>1</v>
       </c>
@@ -2411,16 +2419,16 @@
       <c r="J3">
         <v>2</v>
       </c>
-      <c r="K3" s="41" t="s">
+      <c r="K3" s="40" t="s">
         <v>14</v>
       </c>
-      <c r="L3" s="38">
+      <c r="L3" s="37">
         <v>2</v>
       </c>
-      <c r="M3" s="38">
+      <c r="M3" s="37">
         <v>2</v>
       </c>
-      <c r="N3" s="35" t="s">
+      <c r="N3" s="34" t="s">
         <v>5</v>
       </c>
       <c r="O3" t="s">
@@ -2432,12 +2440,8 @@
       <c r="Q3" s="21">
         <v>24</v>
       </c>
-      <c r="R3">
-        <v>27</v>
-      </c>
-      <c r="S3">
-        <v>30</v>
-      </c>
+      <c r="R3" s="111"/>
+      <c r="S3" s="111"/>
       <c r="T3">
         <f t="shared" si="4"/>
         <v>60</v>
@@ -2458,11 +2462,11 @@
         <f t="shared" si="0"/>
         <v>72</v>
       </c>
-      <c r="Y3" s="54">
+      <c r="Y3" s="53">
         <f t="shared" si="4"/>
         <v>75</v>
       </c>
-      <c r="Z3" s="55">
+      <c r="Z3" s="54">
         <v>5</v>
       </c>
       <c r="AA3">
@@ -2721,16 +2725,16 @@
       <c r="J4">
         <v>2</v>
       </c>
-      <c r="K4" s="42" t="s">
+      <c r="K4" s="41" t="s">
         <v>15</v>
       </c>
-      <c r="L4" s="38">
+      <c r="L4" s="37">
         <v>2</v>
       </c>
-      <c r="M4" s="38">
+      <c r="M4" s="37">
         <v>2</v>
       </c>
-      <c r="N4" s="35" t="s">
+      <c r="N4" s="34" t="s">
         <v>4</v>
       </c>
       <c r="O4" t="s">
@@ -2758,16 +2762,16 @@
         <f t="shared" si="5"/>
         <v>84</v>
       </c>
-      <c r="V4" s="99" t="s">
+      <c r="V4" s="101" t="s">
         <v>33</v>
       </c>
-      <c r="W4" s="100"/>
-      <c r="X4" s="101"/>
-      <c r="Y4" s="54">
+      <c r="W4" s="102"/>
+      <c r="X4" s="103"/>
+      <c r="Y4" s="53">
         <f t="shared" si="4"/>
         <v>100</v>
       </c>
-      <c r="Z4" s="55">
+      <c r="Z4" s="54">
         <v>5</v>
       </c>
       <c r="AB4">
@@ -3022,14 +3026,14 @@
       <c r="J5">
         <v>2</v>
       </c>
-      <c r="K5" s="43" t="s">
+      <c r="K5" s="42" t="s">
         <v>24</v>
       </c>
-      <c r="L5" s="43"/>
-      <c r="M5" s="38">
+      <c r="L5" s="42"/>
+      <c r="M5" s="37">
         <v>2</v>
       </c>
-      <c r="N5" s="35" t="s">
+      <c r="N5" s="34" t="s">
         <v>7</v>
       </c>
       <c r="O5" t="s">
@@ -3055,9 +3059,9 @@
         <f t="shared" si="5"/>
         <v>105</v>
       </c>
-      <c r="V5" s="102"/>
-      <c r="W5" s="103"/>
-      <c r="X5" s="104"/>
+      <c r="V5" s="104"/>
+      <c r="W5" s="105"/>
+      <c r="X5" s="106"/>
       <c r="Y5" s="13">
         <v>62</v>
       </c>
@@ -3302,12 +3306,10 @@
       <c r="D6" s="20">
         <v>1</v>
       </c>
-      <c r="E6" s="20">
-        <v>1</v>
-      </c>
-      <c r="F6" s="20">
-        <v>1</v>
-      </c>
+      <c r="E6" s="110">
+        <v>1</v>
+      </c>
+      <c r="F6" s="110"/>
       <c r="G6" s="20">
         <v>1</v>
       </c>
@@ -3320,12 +3322,12 @@
       <c r="J6">
         <v>12</v>
       </c>
-      <c r="K6" s="43" t="s">
+      <c r="K6" s="42" t="s">
         <v>16</v>
       </c>
-      <c r="L6" s="43"/>
-      <c r="M6" s="43"/>
-      <c r="N6" s="35" t="s">
+      <c r="L6" s="42"/>
+      <c r="M6" s="42"/>
+      <c r="N6" s="34" t="s">
         <v>8</v>
       </c>
       <c r="O6" t="s">
@@ -3351,9 +3353,9 @@
         <f t="shared" si="0"/>
         <v>126</v>
       </c>
-      <c r="V6" s="102"/>
-      <c r="W6" s="103"/>
-      <c r="X6" s="104"/>
+      <c r="V6" s="104"/>
+      <c r="W6" s="105"/>
+      <c r="X6" s="106"/>
       <c r="Y6" s="13">
         <v>0</v>
       </c>
@@ -3598,12 +3600,8 @@
       <c r="D7" s="20">
         <v>1</v>
       </c>
-      <c r="E7" s="20">
-        <v>1</v>
-      </c>
-      <c r="F7" s="20">
-        <v>1</v>
-      </c>
+      <c r="E7" s="110"/>
+      <c r="F7" s="110"/>
       <c r="G7" s="20">
         <v>1</v>
       </c>
@@ -3614,14 +3612,14 @@
         <v>1</v>
       </c>
       <c r="J7" s="23"/>
-      <c r="K7" s="44" t="s">
+      <c r="K7" s="43" t="s">
         <v>17</v>
       </c>
-      <c r="L7" s="45">
+      <c r="L7" s="44">
         <v>33</v>
       </c>
-      <c r="M7" s="45"/>
-      <c r="N7" s="35" t="s">
+      <c r="M7" s="44"/>
+      <c r="N7" s="34" t="s">
         <v>9</v>
       </c>
       <c r="O7" t="s">
@@ -3647,9 +3645,9 @@
         <f t="shared" si="0"/>
         <v>147</v>
       </c>
-      <c r="V7" s="105"/>
-      <c r="W7" s="106"/>
-      <c r="X7" s="107"/>
+      <c r="V7" s="107"/>
+      <c r="W7" s="108"/>
+      <c r="X7" s="109"/>
       <c r="Y7">
         <v>5</v>
       </c>
@@ -3892,12 +3890,8 @@
       <c r="D8" s="20">
         <v>1</v>
       </c>
-      <c r="E8" s="20">
-        <v>1</v>
-      </c>
-      <c r="F8" s="20">
-        <v>1</v>
-      </c>
+      <c r="E8" s="110"/>
+      <c r="F8" s="110"/>
       <c r="G8" s="20">
         <v>1</v>
       </c>
@@ -3908,14 +3902,14 @@
         <v>1</v>
       </c>
       <c r="J8" s="23"/>
-      <c r="K8" s="46" t="s">
+      <c r="K8" s="45" t="s">
         <v>20</v>
       </c>
-      <c r="L8" s="38">
+      <c r="L8" s="37">
         <v>8</v>
       </c>
-      <c r="M8" s="38"/>
-      <c r="N8" s="35" t="s">
+      <c r="M8" s="37"/>
+      <c r="N8" s="34" t="s">
         <v>10</v>
       </c>
       <c r="O8" t="s">
@@ -3927,7 +3921,7 @@
       <c r="Q8" s="19">
         <v>64</v>
       </c>
-      <c r="R8" s="56">
+      <c r="R8" s="55">
         <v>72</v>
       </c>
       <c r="S8">
@@ -4215,14 +4209,14 @@
         <v>1</v>
       </c>
       <c r="J9" s="23"/>
-      <c r="K9" s="47" t="s">
+      <c r="K9" s="46" t="s">
         <v>25</v>
       </c>
-      <c r="L9" s="43"/>
-      <c r="M9" s="38">
+      <c r="L9" s="42"/>
+      <c r="M9" s="37">
         <v>5</v>
       </c>
-      <c r="N9" s="35" t="s">
+      <c r="N9" s="34" t="s">
         <v>11</v>
       </c>
       <c r="O9" t="s">
@@ -4506,12 +4500,10 @@
       <c r="D10" s="20">
         <v>1</v>
       </c>
-      <c r="E10" s="20">
-        <v>1</v>
-      </c>
-      <c r="F10" s="20">
-        <v>1</v>
-      </c>
+      <c r="E10" s="110">
+        <v>1</v>
+      </c>
+      <c r="F10" s="110"/>
       <c r="G10" s="20">
         <v>1</v>
       </c>
@@ -4522,14 +4514,14 @@
         <v>1</v>
       </c>
       <c r="J10" s="23"/>
-      <c r="K10" s="47" t="s">
+      <c r="K10" s="46" t="s">
         <v>18</v>
       </c>
-      <c r="L10" s="38">
+      <c r="L10" s="37">
         <v>4</v>
       </c>
-      <c r="M10" s="38"/>
-      <c r="N10" s="35" t="s">
+      <c r="M10" s="37"/>
+      <c r="N10" s="34" t="s">
         <v>12</v>
       </c>
       <c r="O10" t="s">
@@ -4551,11 +4543,11 @@
         <f t="shared" si="4"/>
         <v>200</v>
       </c>
-      <c r="U10" s="51">
+      <c r="U10" s="50">
         <f t="shared" si="0"/>
         <v>210</v>
       </c>
-      <c r="V10" s="51">
+      <c r="V10" s="50">
         <f t="shared" si="0"/>
         <v>220</v>
       </c>
@@ -4813,12 +4805,8 @@
       <c r="D11" s="20">
         <v>1</v>
       </c>
-      <c r="E11" s="20">
-        <v>1</v>
-      </c>
-      <c r="F11" s="20">
-        <v>1</v>
-      </c>
+      <c r="E11" s="110"/>
+      <c r="F11" s="110"/>
       <c r="G11" s="20">
         <v>1</v>
       </c>
@@ -4831,12 +4819,12 @@
       <c r="J11" s="16">
         <v>3</v>
       </c>
-      <c r="K11" s="47" t="s">
+      <c r="K11" s="46" t="s">
         <v>19</v>
       </c>
-      <c r="L11" s="49"/>
-      <c r="M11" s="48"/>
-      <c r="N11" s="36" t="s">
+      <c r="L11" s="48"/>
+      <c r="M11" s="47"/>
+      <c r="N11" s="35" t="s">
         <v>13</v>
       </c>
       <c r="O11" s="16" t="s">
@@ -4851,16 +4839,16 @@
       <c r="R11" s="16" t="s">
         <v>30</v>
       </c>
-      <c r="S11" s="50" t="s">
+      <c r="S11" s="49" t="s">
         <v>29</v>
       </c>
       <c r="T11" s="16">
         <v>5</v>
       </c>
-      <c r="U11" s="52">
+      <c r="U11" s="51">
         <v>5</v>
       </c>
-      <c r="V11" s="52">
+      <c r="V11" s="51">
         <v>5</v>
       </c>
       <c r="W11" s="16">
@@ -5114,12 +5102,8 @@
       <c r="D12" s="20">
         <v>1</v>
       </c>
-      <c r="E12" s="20">
-        <v>1</v>
-      </c>
-      <c r="F12" s="20">
-        <v>1</v>
-      </c>
+      <c r="E12" s="110"/>
+      <c r="F12" s="110"/>
       <c r="G12" s="20">
         <v>1</v>
       </c>
@@ -5130,12 +5114,12 @@
         <v>1</v>
       </c>
       <c r="J12" s="23"/>
-      <c r="K12" s="47" t="s">
+      <c r="K12" s="46" t="s">
         <v>26</v>
       </c>
-      <c r="L12" s="43"/>
-      <c r="M12" s="43"/>
-      <c r="N12" s="37" t="s">
+      <c r="L12" s="42"/>
+      <c r="M12" s="42"/>
+      <c r="N12" s="36" t="s">
         <v>23</v>
       </c>
       <c r="O12">
@@ -5157,11 +5141,11 @@
         <f t="shared" si="4"/>
         <v>240</v>
       </c>
-      <c r="U12" s="53">
+      <c r="U12" s="52">
         <f t="shared" si="0"/>
         <v>252</v>
       </c>
-      <c r="V12" s="53">
+      <c r="V12" s="52">
         <f t="shared" si="0"/>
         <v>264</v>
       </c>
@@ -5727,12 +5711,10 @@
       <c r="D14" s="20">
         <v>1</v>
       </c>
-      <c r="E14" s="20">
-        <v>1</v>
-      </c>
-      <c r="F14" s="20">
-        <v>1</v>
-      </c>
+      <c r="E14" s="112">
+        <v>1</v>
+      </c>
+      <c r="F14" s="112"/>
       <c r="G14" s="20">
         <v>1</v>
       </c>
@@ -6035,12 +6017,8 @@
       <c r="D15" s="20">
         <v>1</v>
       </c>
-      <c r="E15" s="20">
-        <v>1</v>
-      </c>
-      <c r="F15" s="20">
-        <v>1</v>
-      </c>
+      <c r="E15" s="112"/>
+      <c r="F15" s="112"/>
       <c r="G15" s="20">
         <v>1</v>
       </c>
@@ -6344,12 +6322,8 @@
       <c r="D16" s="20">
         <v>1</v>
       </c>
-      <c r="E16" s="20">
-        <v>1</v>
-      </c>
-      <c r="F16" s="20">
-        <v>1</v>
-      </c>
+      <c r="E16" s="112"/>
+      <c r="F16" s="112"/>
       <c r="G16" s="20">
         <v>1</v>
       </c>
@@ -6362,22 +6336,22 @@
       <c r="J16" s="1">
         <v>32</v>
       </c>
-      <c r="K16" s="79" t="s">
+      <c r="K16" s="78" t="s">
         <v>2</v>
       </c>
-      <c r="L16" s="80"/>
-      <c r="M16" s="80"/>
-      <c r="N16" s="80"/>
-      <c r="O16" s="80"/>
-      <c r="P16" s="80"/>
-      <c r="Q16" s="80"/>
-      <c r="R16" s="80"/>
-      <c r="S16" s="80"/>
-      <c r="T16" s="80"/>
-      <c r="U16" s="80"/>
-      <c r="V16" s="80"/>
-      <c r="W16" s="80"/>
-      <c r="X16" s="81"/>
+      <c r="L16" s="79"/>
+      <c r="M16" s="79"/>
+      <c r="N16" s="79"/>
+      <c r="O16" s="79"/>
+      <c r="P16" s="79"/>
+      <c r="Q16" s="79"/>
+      <c r="R16" s="79"/>
+      <c r="S16" s="79"/>
+      <c r="T16" s="79"/>
+      <c r="U16" s="79"/>
+      <c r="V16" s="79"/>
+      <c r="W16" s="79"/>
+      <c r="X16" s="80"/>
       <c r="Y16">
         <f t="shared" si="4"/>
         <v>400</v>
@@ -6730,7 +6704,7 @@
         <f t="shared" si="4"/>
         <v>595</v>
       </c>
-      <c r="AJ17" s="108">
+      <c r="AJ17" s="98">
         <f t="shared" si="7"/>
         <v>612</v>
       </c>
@@ -7037,7 +7011,7 @@
         <f t="shared" si="4"/>
         <v>630</v>
       </c>
-      <c r="AJ18" s="109"/>
+      <c r="AJ18" s="99"/>
       <c r="AK18">
         <f t="shared" si="7"/>
         <v>666</v>
@@ -7236,13 +7210,13 @@
       <c r="D19" s="20">
         <v>1</v>
       </c>
-      <c r="E19" s="61">
-        <v>1</v>
-      </c>
-      <c r="F19" s="61">
-        <v>1</v>
-      </c>
-      <c r="G19" s="61">
+      <c r="E19" s="60">
+        <v>1</v>
+      </c>
+      <c r="F19" s="60">
+        <v>1</v>
+      </c>
+      <c r="G19" s="60">
         <v>1</v>
       </c>
       <c r="H19" s="20">
@@ -7305,27 +7279,27 @@
         <f t="shared" si="4"/>
         <v>494</v>
       </c>
-      <c r="AA19" s="66">
+      <c r="AA19" s="65">
         <f t="shared" si="4"/>
         <v>513</v>
       </c>
-      <c r="AB19" s="66">
+      <c r="AB19" s="65">
         <f t="shared" si="4"/>
         <v>532</v>
       </c>
-      <c r="AC19" s="66">
+      <c r="AC19" s="65">
         <f t="shared" si="4"/>
         <v>551</v>
       </c>
-      <c r="AD19" s="66">
+      <c r="AD19" s="65">
         <f t="shared" si="4"/>
         <v>570</v>
       </c>
-      <c r="AE19" s="66">
+      <c r="AE19" s="65">
         <f t="shared" si="4"/>
         <v>589</v>
       </c>
-      <c r="AF19" s="66">
+      <c r="AF19" s="65">
         <f t="shared" si="4"/>
         <v>608</v>
       </c>
@@ -7341,7 +7315,7 @@
         <f t="shared" si="4"/>
         <v>665</v>
       </c>
-      <c r="AJ19" s="109"/>
+      <c r="AJ19" s="99"/>
       <c r="AK19">
         <f t="shared" si="7"/>
         <v>703</v>
@@ -7540,13 +7514,13 @@
       <c r="D20" s="20">
         <v>1</v>
       </c>
-      <c r="E20" s="62">
-        <v>1</v>
-      </c>
-      <c r="F20" s="62">
-        <v>1</v>
-      </c>
-      <c r="G20" s="62">
+      <c r="E20" s="61">
+        <v>1</v>
+      </c>
+      <c r="F20" s="61">
+        <v>1</v>
+      </c>
+      <c r="G20" s="61">
         <v>1</v>
       </c>
       <c r="H20" s="20">
@@ -7609,27 +7583,27 @@
       <c r="Z20" t="s">
         <v>33</v>
       </c>
-      <c r="AA20" s="66">
+      <c r="AA20" s="65">
         <f t="shared" si="4"/>
         <v>540</v>
       </c>
-      <c r="AB20" s="66">
+      <c r="AB20" s="65">
         <f t="shared" si="4"/>
         <v>560</v>
       </c>
-      <c r="AC20" s="67">
+      <c r="AC20" s="66">
         <f t="shared" si="4"/>
         <v>580</v>
       </c>
-      <c r="AD20" s="68">
+      <c r="AD20" s="67">
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="AE20" s="69">
+      <c r="AE20" s="68">
         <f t="shared" si="4"/>
         <v>620</v>
       </c>
-      <c r="AF20" s="66">
+      <c r="AF20" s="65">
         <f t="shared" si="4"/>
         <v>640</v>
       </c>
@@ -7645,7 +7619,7 @@
         <f t="shared" si="4"/>
         <v>700</v>
       </c>
-      <c r="AJ20" s="109"/>
+      <c r="AJ20" s="99"/>
       <c r="AK20">
         <f t="shared" si="7"/>
         <v>740</v>
@@ -7844,16 +7818,16 @@
       <c r="D21" s="20">
         <v>1</v>
       </c>
-      <c r="E21" s="63">
-        <v>1</v>
-      </c>
-      <c r="F21" s="63">
-        <v>1</v>
-      </c>
-      <c r="G21" s="63">
-        <v>1</v>
-      </c>
-      <c r="H21" s="65">
+      <c r="E21" s="62">
+        <v>1</v>
+      </c>
+      <c r="F21" s="62">
+        <v>1</v>
+      </c>
+      <c r="G21" s="62">
+        <v>1</v>
+      </c>
+      <c r="H21" s="64">
         <v>1</v>
       </c>
       <c r="I21" s="20">
@@ -7883,10 +7857,10 @@
       <c r="R21">
         <v>189</v>
       </c>
-      <c r="S21" s="59">
+      <c r="S21" s="58">
         <v>210</v>
       </c>
-      <c r="T21" s="60">
+      <c r="T21" s="59">
         <f t="shared" si="4"/>
         <v>420</v>
       </c>
@@ -7894,7 +7868,7 @@
         <f t="shared" si="4"/>
         <v>441</v>
       </c>
-      <c r="V21" s="51">
+      <c r="V21" s="50">
         <f t="shared" si="4"/>
         <v>462</v>
       </c>
@@ -7902,7 +7876,7 @@
         <f t="shared" si="4"/>
         <v>483</v>
       </c>
-      <c r="X21" s="51">
+      <c r="X21" s="50">
         <f t="shared" si="4"/>
         <v>504</v>
       </c>
@@ -7914,27 +7888,27 @@
         <f t="shared" si="4"/>
         <v>546</v>
       </c>
-      <c r="AA21" s="66">
+      <c r="AA21" s="65">
         <f t="shared" si="4"/>
         <v>567</v>
       </c>
-      <c r="AB21" s="66">
+      <c r="AB21" s="65">
         <f t="shared" si="4"/>
         <v>588</v>
       </c>
-      <c r="AC21" s="70">
+      <c r="AC21" s="69">
         <f t="shared" si="4"/>
         <v>609</v>
       </c>
-      <c r="AD21" s="77">
+      <c r="AD21" s="76">
         <f t="shared" si="4"/>
         <v>630</v>
       </c>
-      <c r="AE21" s="71">
+      <c r="AE21" s="70">
         <f t="shared" si="4"/>
         <v>651</v>
       </c>
-      <c r="AF21" s="66">
+      <c r="AF21" s="65">
         <f t="shared" si="4"/>
         <v>672</v>
       </c>
@@ -7950,7 +7924,7 @@
         <f t="shared" si="4"/>
         <v>735</v>
       </c>
-      <c r="AJ21" s="109"/>
+      <c r="AJ21" s="99"/>
       <c r="AK21">
         <f t="shared" si="7"/>
         <v>777</v>
@@ -8149,13 +8123,13 @@
       <c r="D22" s="20">
         <v>1</v>
       </c>
-      <c r="E22" s="64">
-        <v>1</v>
-      </c>
-      <c r="F22" s="64">
-        <v>1</v>
-      </c>
-      <c r="G22" s="64">
+      <c r="E22" s="63">
+        <v>1</v>
+      </c>
+      <c r="F22" s="63">
+        <v>1</v>
+      </c>
+      <c r="G22" s="63">
         <v>1</v>
       </c>
       <c r="H22" s="20">
@@ -8167,12 +8141,12 @@
       <c r="J22">
         <v>44</v>
       </c>
-      <c r="K22" s="82" t="s">
+      <c r="K22" s="81" t="s">
         <v>0</v>
       </c>
-      <c r="L22" s="83"/>
-      <c r="M22" s="83"/>
-      <c r="N22" s="84"/>
+      <c r="L22" s="82"/>
+      <c r="M22" s="82"/>
+      <c r="N22" s="83"/>
       <c r="O22">
         <v>132</v>
       </c>
@@ -8185,14 +8159,14 @@
       <c r="R22">
         <v>198</v>
       </c>
-      <c r="S22" s="91" t="s">
-        <v>1</v>
-      </c>
-      <c r="T22" s="92"/>
-      <c r="U22" s="93"/>
-      <c r="V22" s="92"/>
-      <c r="W22" s="93"/>
-      <c r="X22" s="94"/>
+      <c r="S22" s="90" t="s">
+        <v>1</v>
+      </c>
+      <c r="T22" s="91"/>
+      <c r="U22" s="92"/>
+      <c r="V22" s="91"/>
+      <c r="W22" s="92"/>
+      <c r="X22" s="93"/>
       <c r="Y22">
         <f t="shared" si="4"/>
         <v>550</v>
@@ -8201,27 +8175,27 @@
         <f t="shared" si="4"/>
         <v>572</v>
       </c>
-      <c r="AA22" s="66">
+      <c r="AA22" s="65">
         <f t="shared" si="4"/>
         <v>594</v>
       </c>
-      <c r="AB22" s="66">
+      <c r="AB22" s="65">
         <f t="shared" si="4"/>
         <v>616</v>
       </c>
-      <c r="AC22" s="70">
+      <c r="AC22" s="69">
         <f t="shared" si="4"/>
         <v>638</v>
       </c>
-      <c r="AD22" s="75">
+      <c r="AD22" s="74">
         <f t="shared" si="4"/>
         <v>660</v>
       </c>
-      <c r="AE22" s="71">
+      <c r="AE22" s="70">
         <f t="shared" si="4"/>
         <v>682</v>
       </c>
-      <c r="AF22" s="66">
+      <c r="AF22" s="65">
         <f t="shared" si="4"/>
         <v>704</v>
       </c>
@@ -8237,7 +8211,7 @@
         <f t="shared" si="4"/>
         <v>770</v>
       </c>
-      <c r="AJ22" s="109"/>
+      <c r="AJ22" s="99"/>
       <c r="AK22">
         <f t="shared" si="7"/>
         <v>814</v>
@@ -8456,10 +8430,10 @@
         <f t="shared" si="10"/>
         <v>230</v>
       </c>
-      <c r="K23" s="85"/>
-      <c r="L23" s="86"/>
-      <c r="M23" s="86"/>
-      <c r="N23" s="87"/>
+      <c r="K23" s="84"/>
+      <c r="L23" s="85"/>
+      <c r="M23" s="85"/>
+      <c r="N23" s="86"/>
       <c r="O23">
         <f t="shared" si="10"/>
         <v>345</v>
@@ -8476,12 +8450,12 @@
         <f t="shared" si="10"/>
         <v>414</v>
       </c>
-      <c r="S23" s="95"/>
-      <c r="T23" s="92"/>
-      <c r="U23" s="92"/>
-      <c r="V23" s="92"/>
-      <c r="W23" s="92"/>
-      <c r="X23" s="94"/>
+      <c r="S23" s="94"/>
+      <c r="T23" s="91"/>
+      <c r="U23" s="91"/>
+      <c r="V23" s="91"/>
+      <c r="W23" s="91"/>
+      <c r="X23" s="93"/>
       <c r="Y23">
         <f t="shared" si="4"/>
         <v>575</v>
@@ -8490,27 +8464,27 @@
         <f t="shared" si="4"/>
         <v>598</v>
       </c>
-      <c r="AA23" s="66">
+      <c r="AA23" s="65">
         <f t="shared" si="4"/>
         <v>621</v>
       </c>
-      <c r="AB23" s="66">
+      <c r="AB23" s="65">
         <f t="shared" si="4"/>
         <v>644</v>
       </c>
-      <c r="AC23" s="70">
+      <c r="AC23" s="69">
         <f t="shared" si="4"/>
         <v>667</v>
       </c>
-      <c r="AD23" s="76">
+      <c r="AD23" s="75">
         <f t="shared" si="4"/>
         <v>690</v>
       </c>
-      <c r="AE23" s="71">
+      <c r="AE23" s="70">
         <f t="shared" si="4"/>
         <v>713</v>
       </c>
-      <c r="AF23" s="66">
+      <c r="AF23" s="65">
         <f t="shared" si="4"/>
         <v>736</v>
       </c>
@@ -8526,7 +8500,7 @@
         <f t="shared" si="4"/>
         <v>805</v>
       </c>
-      <c r="AJ23" s="109"/>
+      <c r="AJ23" s="99"/>
       <c r="AK23">
         <f t="shared" si="7"/>
         <v>851</v>
@@ -8745,10 +8719,10 @@
         <f t="shared" si="10"/>
         <v>240</v>
       </c>
-      <c r="K24" s="88"/>
-      <c r="L24" s="89"/>
-      <c r="M24" s="89"/>
-      <c r="N24" s="90"/>
+      <c r="K24" s="87"/>
+      <c r="L24" s="88"/>
+      <c r="M24" s="88"/>
+      <c r="N24" s="89"/>
       <c r="O24">
         <f t="shared" si="10"/>
         <v>360</v>
@@ -8765,12 +8739,12 @@
         <f t="shared" si="10"/>
         <v>432</v>
       </c>
-      <c r="S24" s="96"/>
-      <c r="T24" s="92"/>
-      <c r="U24" s="97"/>
-      <c r="V24" s="92"/>
-      <c r="W24" s="97"/>
-      <c r="X24" s="98"/>
+      <c r="S24" s="95"/>
+      <c r="T24" s="91"/>
+      <c r="U24" s="96"/>
+      <c r="V24" s="91"/>
+      <c r="W24" s="96"/>
+      <c r="X24" s="97"/>
       <c r="Y24">
         <f t="shared" si="4"/>
         <v>600</v>
@@ -8779,27 +8753,27 @@
         <f t="shared" si="4"/>
         <v>624</v>
       </c>
-      <c r="AA24" s="66">
+      <c r="AA24" s="65">
         <f t="shared" si="4"/>
         <v>648</v>
       </c>
-      <c r="AB24" s="66">
+      <c r="AB24" s="65">
         <f t="shared" si="4"/>
         <v>672</v>
       </c>
-      <c r="AC24" s="70">
+      <c r="AC24" s="69">
         <f t="shared" si="4"/>
         <v>696</v>
       </c>
-      <c r="AD24" s="76">
+      <c r="AD24" s="75">
         <f t="shared" si="4"/>
         <v>720</v>
       </c>
-      <c r="AE24" s="71">
+      <c r="AE24" s="70">
         <f t="shared" si="4"/>
         <v>744</v>
       </c>
-      <c r="AF24" s="66">
+      <c r="AF24" s="65">
         <f t="shared" si="4"/>
         <v>768</v>
       </c>
@@ -8815,7 +8789,7 @@
         <f t="shared" si="4"/>
         <v>840</v>
       </c>
-      <c r="AJ24" s="109"/>
+      <c r="AJ24" s="99"/>
       <c r="AK24">
         <f t="shared" si="7"/>
         <v>888</v>
@@ -9066,7 +9040,7 @@
         <f t="shared" si="10"/>
         <v>475</v>
       </c>
-      <c r="T25" s="57">
+      <c r="T25" s="56">
         <f t="shared" si="4"/>
         <v>500</v>
       </c>
@@ -9074,7 +9048,7 @@
         <f t="shared" si="4"/>
         <v>525</v>
       </c>
-      <c r="V25" s="57">
+      <c r="V25" s="56">
         <f t="shared" si="4"/>
         <v>550</v>
       </c>
@@ -9094,27 +9068,27 @@
         <f t="shared" si="4"/>
         <v>650</v>
       </c>
-      <c r="AA25" s="66">
+      <c r="AA25" s="65">
         <f t="shared" si="4"/>
         <v>675</v>
       </c>
-      <c r="AB25" s="66">
+      <c r="AB25" s="65">
         <f t="shared" si="4"/>
         <v>700</v>
       </c>
-      <c r="AC25" s="70">
+      <c r="AC25" s="69">
         <f t="shared" si="4"/>
         <v>725</v>
       </c>
-      <c r="AD25" s="76">
+      <c r="AD25" s="75">
         <f t="shared" si="4"/>
         <v>750</v>
       </c>
-      <c r="AE25" s="71">
+      <c r="AE25" s="70">
         <f t="shared" si="4"/>
         <v>775</v>
       </c>
-      <c r="AF25" s="66">
+      <c r="AF25" s="65">
         <f t="shared" si="4"/>
         <v>800</v>
       </c>
@@ -9130,7 +9104,7 @@
         <f t="shared" si="4"/>
         <v>875</v>
       </c>
-      <c r="AJ25" s="109"/>
+      <c r="AJ25" s="99"/>
       <c r="AK25">
         <f t="shared" si="7"/>
         <v>925</v>
@@ -9409,27 +9383,27 @@
         <f t="shared" si="4"/>
         <v>676</v>
       </c>
-      <c r="AA26" s="66">
+      <c r="AA26" s="65">
         <f t="shared" si="4"/>
         <v>702</v>
       </c>
-      <c r="AB26" s="66">
+      <c r="AB26" s="65">
         <f t="shared" si="4"/>
         <v>728</v>
       </c>
-      <c r="AC26" s="70">
+      <c r="AC26" s="69">
         <f t="shared" si="4"/>
         <v>754</v>
       </c>
-      <c r="AD26" s="75">
+      <c r="AD26" s="74">
         <f t="shared" si="4"/>
         <v>780</v>
       </c>
-      <c r="AE26" s="71">
+      <c r="AE26" s="70">
         <f t="shared" si="4"/>
         <v>806</v>
       </c>
-      <c r="AF26" s="66">
+      <c r="AF26" s="65">
         <f t="shared" si="4"/>
         <v>832</v>
       </c>
@@ -9445,7 +9419,7 @@
         <f t="shared" si="4"/>
         <v>910</v>
       </c>
-      <c r="AJ26" s="109"/>
+      <c r="AJ26" s="99"/>
       <c r="AK26">
         <f t="shared" si="7"/>
         <v>962</v>
@@ -9672,23 +9646,23 @@
         <f t="shared" si="10"/>
         <v>324</v>
       </c>
-      <c r="N27" s="58">
+      <c r="N27" s="57">
         <f t="shared" si="10"/>
         <v>378</v>
       </c>
-      <c r="O27" s="58">
+      <c r="O27" s="57">
         <f t="shared" si="10"/>
         <v>405</v>
       </c>
-      <c r="P27" s="58">
+      <c r="P27" s="57">
         <f t="shared" si="10"/>
         <v>432</v>
       </c>
-      <c r="Q27" s="58">
+      <c r="Q27" s="57">
         <f t="shared" si="10"/>
         <v>459</v>
       </c>
-      <c r="R27" s="58">
+      <c r="R27" s="57">
         <f t="shared" si="10"/>
         <v>486</v>
       </c>
@@ -9724,27 +9698,27 @@
         <f t="shared" si="4"/>
         <v>702</v>
       </c>
-      <c r="AA27" s="66">
+      <c r="AA27" s="65">
         <f t="shared" si="4"/>
         <v>729</v>
       </c>
-      <c r="AB27" s="66">
+      <c r="AB27" s="65">
         <f t="shared" si="4"/>
         <v>756</v>
       </c>
-      <c r="AC27" s="70">
+      <c r="AC27" s="69">
         <f t="shared" si="4"/>
         <v>783</v>
       </c>
-      <c r="AD27" s="78">
+      <c r="AD27" s="77">
         <f t="shared" si="4"/>
         <v>810</v>
       </c>
-      <c r="AE27" s="71">
+      <c r="AE27" s="70">
         <f t="shared" si="4"/>
         <v>837</v>
       </c>
-      <c r="AF27" s="66">
+      <c r="AF27" s="65">
         <f t="shared" si="4"/>
         <v>864</v>
       </c>
@@ -9760,7 +9734,7 @@
         <f t="shared" si="4"/>
         <v>945</v>
       </c>
-      <c r="AJ27" s="109"/>
+      <c r="AJ27" s="99"/>
       <c r="AK27">
         <f t="shared" si="7"/>
         <v>999</v>
@@ -9987,23 +9961,23 @@
         <f t="shared" si="10"/>
         <v>336</v>
       </c>
-      <c r="N28" s="58">
+      <c r="N28" s="57">
         <f t="shared" si="10"/>
         <v>392</v>
       </c>
-      <c r="O28" s="58">
+      <c r="O28" s="57">
         <f t="shared" si="10"/>
         <v>420</v>
       </c>
-      <c r="P28" s="58">
+      <c r="P28" s="57">
         <f t="shared" si="10"/>
         <v>448</v>
       </c>
-      <c r="Q28" s="58">
+      <c r="Q28" s="57">
         <f t="shared" si="10"/>
         <v>476</v>
       </c>
-      <c r="R28" s="58">
+      <c r="R28" s="57">
         <f t="shared" si="10"/>
         <v>504</v>
       </c>
@@ -10039,27 +10013,27 @@
         <f t="shared" si="4"/>
         <v>728</v>
       </c>
-      <c r="AA28" s="66">
+      <c r="AA28" s="65">
         <f t="shared" si="4"/>
         <v>756</v>
       </c>
-      <c r="AB28" s="66">
+      <c r="AB28" s="65">
         <f t="shared" si="4"/>
         <v>784</v>
       </c>
-      <c r="AC28" s="72">
+      <c r="AC28" s="71">
         <f t="shared" si="4"/>
         <v>812</v>
       </c>
-      <c r="AD28" s="73">
+      <c r="AD28" s="72">
         <f t="shared" si="4"/>
         <v>840</v>
       </c>
-      <c r="AE28" s="74">
+      <c r="AE28" s="73">
         <f t="shared" si="4"/>
         <v>868</v>
       </c>
-      <c r="AF28" s="66">
+      <c r="AF28" s="65">
         <f t="shared" si="4"/>
         <v>896</v>
       </c>
@@ -10075,7 +10049,7 @@
         <f t="shared" si="4"/>
         <v>980</v>
       </c>
-      <c r="AJ28" s="110"/>
+      <c r="AJ28" s="100"/>
       <c r="AK28">
         <f t="shared" si="7"/>
         <v>1036</v>
@@ -10112,50 +10086,20 @@
         <f t="shared" si="7"/>
         <v>1260</v>
       </c>
-      <c r="AT28">
+      <c r="AT28" s="114">
         <f t="shared" si="7"/>
         <v>1288</v>
       </c>
-      <c r="AU28">
-        <f t="shared" si="8"/>
-        <v>1316</v>
-      </c>
-      <c r="AV28">
-        <f t="shared" si="8"/>
-        <v>1344</v>
-      </c>
-      <c r="AW28">
-        <f t="shared" si="8"/>
-        <v>1372</v>
-      </c>
-      <c r="AX28">
-        <f t="shared" si="8"/>
-        <v>1400</v>
-      </c>
-      <c r="AY28">
-        <f t="shared" si="8"/>
-        <v>1428</v>
-      </c>
-      <c r="AZ28">
-        <f t="shared" si="8"/>
-        <v>1456</v>
-      </c>
-      <c r="BA28">
-        <f t="shared" si="8"/>
-        <v>1484</v>
-      </c>
-      <c r="BB28">
-        <f t="shared" si="8"/>
-        <v>1512</v>
-      </c>
-      <c r="BC28">
-        <f t="shared" si="8"/>
-        <v>1540</v>
-      </c>
-      <c r="BD28">
-        <f t="shared" si="8"/>
-        <v>1568</v>
-      </c>
+      <c r="AU28" s="114"/>
+      <c r="AV28" s="114"/>
+      <c r="AW28" s="114"/>
+      <c r="AX28" s="114"/>
+      <c r="AY28" s="114"/>
+      <c r="AZ28" s="114"/>
+      <c r="BA28" s="114"/>
+      <c r="BB28" s="114"/>
+      <c r="BC28" s="114"/>
+      <c r="BD28" s="114"/>
       <c r="BE28">
         <f t="shared" si="8"/>
         <v>1596</v>
@@ -10302,23 +10246,23 @@
         <f t="shared" si="10"/>
         <v>348</v>
       </c>
-      <c r="N29" s="58">
+      <c r="N29" s="57">
         <f t="shared" si="10"/>
         <v>406</v>
       </c>
-      <c r="O29" s="58">
+      <c r="O29" s="57">
         <f t="shared" si="10"/>
         <v>435</v>
       </c>
-      <c r="P29" s="58">
+      <c r="P29" s="57">
         <f t="shared" si="10"/>
         <v>464</v>
       </c>
-      <c r="Q29" s="58">
+      <c r="Q29" s="57">
         <f t="shared" si="10"/>
         <v>493</v>
       </c>
-      <c r="R29" s="58">
+      <c r="R29" s="57">
         <f t="shared" si="10"/>
         <v>522</v>
       </c>
@@ -10351,27 +10295,27 @@
         <f t="shared" si="4"/>
         <v>754</v>
       </c>
-      <c r="AA29" s="66">
+      <c r="AA29" s="65">
         <f t="shared" si="4"/>
         <v>783</v>
       </c>
-      <c r="AB29" s="66">
+      <c r="AB29" s="65">
         <f t="shared" si="4"/>
         <v>812</v>
       </c>
-      <c r="AC29" s="66">
+      <c r="AC29" s="65">
         <f t="shared" si="4"/>
         <v>841</v>
       </c>
-      <c r="AD29" s="66">
+      <c r="AD29" s="65">
         <f t="shared" si="4"/>
         <v>870</v>
       </c>
-      <c r="AE29" s="66">
+      <c r="AE29" s="65">
         <f t="shared" si="4"/>
         <v>899</v>
       </c>
-      <c r="AF29" s="66">
+      <c r="AF29" s="65">
         <f t="shared" si="4"/>
         <v>928</v>
       </c>
@@ -10427,50 +10371,17 @@
         <f t="shared" si="7"/>
         <v>1305</v>
       </c>
-      <c r="AT29">
-        <f t="shared" si="7"/>
-        <v>1334</v>
-      </c>
-      <c r="AU29">
-        <f t="shared" si="8"/>
-        <v>1363</v>
-      </c>
-      <c r="AV29">
-        <f t="shared" si="8"/>
-        <v>1392</v>
-      </c>
-      <c r="AW29">
-        <f t="shared" si="8"/>
-        <v>1421</v>
-      </c>
-      <c r="AX29">
-        <f t="shared" si="8"/>
-        <v>1450</v>
-      </c>
-      <c r="AY29">
-        <f t="shared" si="8"/>
-        <v>1479</v>
-      </c>
-      <c r="AZ29">
-        <f t="shared" si="8"/>
-        <v>1508</v>
-      </c>
-      <c r="BA29">
-        <f t="shared" si="8"/>
-        <v>1537</v>
-      </c>
-      <c r="BB29">
-        <f t="shared" si="8"/>
-        <v>1566</v>
-      </c>
-      <c r="BC29">
-        <f t="shared" si="8"/>
-        <v>1595</v>
-      </c>
-      <c r="BD29">
-        <f t="shared" si="8"/>
-        <v>1624</v>
-      </c>
+      <c r="AT29" s="114"/>
+      <c r="AU29" s="114"/>
+      <c r="AV29" s="114"/>
+      <c r="AW29" s="114"/>
+      <c r="AX29" s="114"/>
+      <c r="AY29" s="114"/>
+      <c r="AZ29" s="114"/>
+      <c r="BA29" s="114"/>
+      <c r="BB29" s="114"/>
+      <c r="BC29" s="114"/>
+      <c r="BD29" s="114"/>
       <c r="BE29">
         <f t="shared" si="8"/>
         <v>1653</v>
@@ -10641,11 +10552,11 @@
         <f t="shared" si="10"/>
         <v>570</v>
       </c>
-      <c r="T30">
+      <c r="T30" s="1">
         <f t="shared" si="4"/>
         <v>600</v>
       </c>
-      <c r="U30" s="33">
+      <c r="U30" s="1">
         <f t="shared" si="4"/>
         <v>630</v>
       </c>
@@ -10745,50 +10656,17 @@
         <f t="shared" si="7"/>
         <v>1350</v>
       </c>
-      <c r="AT30">
-        <f t="shared" si="7"/>
-        <v>1380</v>
-      </c>
-      <c r="AU30">
-        <f t="shared" si="8"/>
-        <v>1410</v>
-      </c>
-      <c r="AV30">
-        <f t="shared" si="8"/>
-        <v>1440</v>
-      </c>
-      <c r="AW30">
-        <f t="shared" si="8"/>
-        <v>1470</v>
-      </c>
-      <c r="AX30">
-        <f t="shared" si="8"/>
-        <v>1500</v>
-      </c>
-      <c r="AY30">
-        <f t="shared" si="8"/>
-        <v>1530</v>
-      </c>
-      <c r="AZ30">
-        <f t="shared" si="8"/>
-        <v>1560</v>
-      </c>
-      <c r="BA30">
-        <f t="shared" si="8"/>
-        <v>1590</v>
-      </c>
-      <c r="BB30">
-        <f t="shared" si="8"/>
-        <v>1620</v>
-      </c>
-      <c r="BC30">
-        <f t="shared" si="8"/>
-        <v>1650</v>
-      </c>
-      <c r="BD30">
-        <f t="shared" si="8"/>
-        <v>1680</v>
-      </c>
+      <c r="AT30" s="114"/>
+      <c r="AU30" s="114"/>
+      <c r="AV30" s="114"/>
+      <c r="AW30" s="114"/>
+      <c r="AX30" s="114"/>
+      <c r="AY30" s="114"/>
+      <c r="AZ30" s="114"/>
+      <c r="BA30" s="114"/>
+      <c r="BB30" s="114"/>
+      <c r="BC30" s="114"/>
+      <c r="BD30" s="114"/>
       <c r="BE30">
         <f t="shared" si="8"/>
         <v>1710</v>
@@ -11063,50 +10941,17 @@
         <f t="shared" si="7"/>
         <v>1395</v>
       </c>
-      <c r="AT31">
-        <f t="shared" si="7"/>
-        <v>1426</v>
-      </c>
-      <c r="AU31">
-        <f t="shared" si="8"/>
-        <v>1457</v>
-      </c>
-      <c r="AV31">
-        <f t="shared" si="8"/>
-        <v>1488</v>
-      </c>
-      <c r="AW31">
-        <f t="shared" si="8"/>
-        <v>1519</v>
-      </c>
-      <c r="AX31">
-        <f t="shared" si="8"/>
-        <v>1550</v>
-      </c>
-      <c r="AY31">
-        <f t="shared" si="8"/>
-        <v>1581</v>
-      </c>
-      <c r="AZ31">
-        <f t="shared" si="8"/>
-        <v>1612</v>
-      </c>
-      <c r="BA31">
-        <f t="shared" si="8"/>
-        <v>1643</v>
-      </c>
-      <c r="BB31">
-        <f t="shared" si="8"/>
-        <v>1674</v>
-      </c>
-      <c r="BC31">
-        <f t="shared" si="8"/>
-        <v>1705</v>
-      </c>
-      <c r="BD31">
-        <f t="shared" si="8"/>
-        <v>1736</v>
-      </c>
+      <c r="AT31" s="114"/>
+      <c r="AU31" s="114"/>
+      <c r="AV31" s="114"/>
+      <c r="AW31" s="114"/>
+      <c r="AX31" s="114"/>
+      <c r="AY31" s="114"/>
+      <c r="AZ31" s="114"/>
+      <c r="BA31" s="114"/>
+      <c r="BB31" s="114"/>
+      <c r="BC31" s="114"/>
+      <c r="BD31" s="114"/>
       <c r="BE31">
         <f t="shared" si="8"/>
         <v>1767</v>
@@ -11381,50 +11226,17 @@
         <f t="shared" si="7"/>
         <v>1440</v>
       </c>
-      <c r="AT32">
-        <f t="shared" si="7"/>
-        <v>1472</v>
-      </c>
-      <c r="AU32">
-        <f t="shared" si="8"/>
-        <v>1504</v>
-      </c>
-      <c r="AV32">
-        <f t="shared" si="8"/>
-        <v>1536</v>
-      </c>
-      <c r="AW32">
-        <f t="shared" si="8"/>
-        <v>1568</v>
-      </c>
-      <c r="AX32">
-        <f t="shared" si="8"/>
-        <v>1600</v>
-      </c>
-      <c r="AY32">
-        <f t="shared" si="8"/>
-        <v>1632</v>
-      </c>
-      <c r="AZ32">
-        <f t="shared" si="8"/>
-        <v>1664</v>
-      </c>
-      <c r="BA32">
-        <f t="shared" si="8"/>
-        <v>1696</v>
-      </c>
-      <c r="BB32">
-        <f t="shared" si="8"/>
-        <v>1728</v>
-      </c>
-      <c r="BC32">
-        <f t="shared" si="8"/>
-        <v>1760</v>
-      </c>
-      <c r="BD32">
-        <f t="shared" si="8"/>
-        <v>1792</v>
-      </c>
+      <c r="AT32" s="114"/>
+      <c r="AU32" s="114"/>
+      <c r="AV32" s="114"/>
+      <c r="AW32" s="114"/>
+      <c r="AX32" s="114"/>
+      <c r="AY32" s="114"/>
+      <c r="AZ32" s="114"/>
+      <c r="BA32" s="114"/>
+      <c r="BB32" s="114"/>
+      <c r="BC32" s="114"/>
+      <c r="BD32" s="114"/>
       <c r="BE32">
         <f t="shared" si="8"/>
         <v>1824</v>
@@ -11680,7 +11492,7 @@
         <v>1320</v>
       </c>
       <c r="AO33">
-        <f t="shared" ref="AO33:BD79" si="14">ROW()*COLUMN()</f>
+        <f t="shared" ref="AO33:BD46" si="14">ROW()*COLUMN()</f>
         <v>1353</v>
       </c>
       <c r="AP33">
@@ -11699,52 +11511,19 @@
         <f t="shared" si="14"/>
         <v>1485</v>
       </c>
-      <c r="AT33">
-        <f t="shared" si="14"/>
-        <v>1518</v>
-      </c>
-      <c r="AU33">
-        <f t="shared" si="14"/>
-        <v>1551</v>
-      </c>
-      <c r="AV33">
-        <f t="shared" si="14"/>
-        <v>1584</v>
-      </c>
-      <c r="AW33">
-        <f t="shared" si="14"/>
-        <v>1617</v>
-      </c>
-      <c r="AX33">
-        <f t="shared" si="14"/>
-        <v>1650</v>
-      </c>
-      <c r="AY33">
-        <f t="shared" si="14"/>
-        <v>1683</v>
-      </c>
-      <c r="AZ33">
-        <f t="shared" si="14"/>
-        <v>1716</v>
-      </c>
-      <c r="BA33">
-        <f t="shared" si="14"/>
-        <v>1749</v>
-      </c>
-      <c r="BB33">
-        <f t="shared" si="14"/>
-        <v>1782</v>
-      </c>
-      <c r="BC33">
-        <f t="shared" si="14"/>
-        <v>1815</v>
-      </c>
-      <c r="BD33">
-        <f t="shared" si="14"/>
-        <v>1848</v>
-      </c>
+      <c r="AT33" s="114"/>
+      <c r="AU33" s="114"/>
+      <c r="AV33" s="114"/>
+      <c r="AW33" s="114"/>
+      <c r="AX33" s="114"/>
+      <c r="AY33" s="114"/>
+      <c r="AZ33" s="114"/>
+      <c r="BA33" s="114"/>
+      <c r="BB33" s="114"/>
+      <c r="BC33" s="114"/>
+      <c r="BD33" s="114"/>
       <c r="BE33">
-        <f t="shared" ref="AU33:BH79" si="15">ROW()*COLUMN()</f>
+        <f t="shared" ref="AU33:BH51" si="15">ROW()*COLUMN()</f>
         <v>1881</v>
       </c>
       <c r="BF33">
@@ -12017,50 +11796,17 @@
         <f t="shared" si="14"/>
         <v>1530</v>
       </c>
-      <c r="AT34">
-        <f t="shared" si="14"/>
-        <v>1564</v>
-      </c>
-      <c r="AU34">
-        <f t="shared" si="15"/>
-        <v>1598</v>
-      </c>
-      <c r="AV34">
-        <f t="shared" si="15"/>
-        <v>1632</v>
-      </c>
-      <c r="AW34">
-        <f t="shared" si="15"/>
-        <v>1666</v>
-      </c>
-      <c r="AX34">
-        <f t="shared" si="15"/>
-        <v>1700</v>
-      </c>
-      <c r="AY34">
-        <f t="shared" si="15"/>
-        <v>1734</v>
-      </c>
-      <c r="AZ34">
-        <f t="shared" si="15"/>
-        <v>1768</v>
-      </c>
-      <c r="BA34">
-        <f t="shared" si="15"/>
-        <v>1802</v>
-      </c>
-      <c r="BB34">
-        <f t="shared" si="15"/>
-        <v>1836</v>
-      </c>
-      <c r="BC34">
-        <f t="shared" si="15"/>
-        <v>1870</v>
-      </c>
-      <c r="BD34">
-        <f t="shared" si="15"/>
-        <v>1904</v>
-      </c>
+      <c r="AT34" s="114"/>
+      <c r="AU34" s="114"/>
+      <c r="AV34" s="114"/>
+      <c r="AW34" s="114"/>
+      <c r="AX34" s="114"/>
+      <c r="AY34" s="114"/>
+      <c r="AZ34" s="114"/>
+      <c r="BA34" s="114"/>
+      <c r="BB34" s="114"/>
+      <c r="BC34" s="114"/>
+      <c r="BD34" s="114"/>
       <c r="BE34">
         <f t="shared" si="15"/>
         <v>1938</v>
@@ -12335,50 +12081,17 @@
         <f t="shared" si="14"/>
         <v>1575</v>
       </c>
-      <c r="AT35">
-        <f t="shared" si="14"/>
-        <v>1610</v>
-      </c>
-      <c r="AU35">
-        <f t="shared" si="15"/>
-        <v>1645</v>
-      </c>
-      <c r="AV35">
-        <f t="shared" si="15"/>
-        <v>1680</v>
-      </c>
-      <c r="AW35">
-        <f t="shared" si="15"/>
-        <v>1715</v>
-      </c>
-      <c r="AX35">
-        <f t="shared" si="15"/>
-        <v>1750</v>
-      </c>
-      <c r="AY35">
-        <f t="shared" si="15"/>
-        <v>1785</v>
-      </c>
-      <c r="AZ35">
-        <f t="shared" si="15"/>
-        <v>1820</v>
-      </c>
-      <c r="BA35">
-        <f t="shared" si="15"/>
-        <v>1855</v>
-      </c>
-      <c r="BB35">
-        <f t="shared" si="15"/>
-        <v>1890</v>
-      </c>
-      <c r="BC35">
-        <f t="shared" si="15"/>
-        <v>1925</v>
-      </c>
-      <c r="BD35">
-        <f t="shared" si="15"/>
-        <v>1960</v>
-      </c>
+      <c r="AT35" s="114"/>
+      <c r="AU35" s="114"/>
+      <c r="AV35" s="114"/>
+      <c r="AW35" s="114"/>
+      <c r="AX35" s="114"/>
+      <c r="AY35" s="114"/>
+      <c r="AZ35" s="114"/>
+      <c r="BA35" s="114"/>
+      <c r="BB35" s="114"/>
+      <c r="BC35" s="114"/>
+      <c r="BD35" s="114"/>
       <c r="BE35">
         <f t="shared" si="15"/>
         <v>1995</v>
@@ -12653,50 +12366,17 @@
         <f t="shared" si="14"/>
         <v>1620</v>
       </c>
-      <c r="AT36">
-        <f t="shared" si="14"/>
-        <v>1656</v>
-      </c>
-      <c r="AU36">
-        <f t="shared" si="15"/>
-        <v>1692</v>
-      </c>
-      <c r="AV36">
-        <f t="shared" si="15"/>
-        <v>1728</v>
-      </c>
-      <c r="AW36">
-        <f t="shared" si="15"/>
-        <v>1764</v>
-      </c>
-      <c r="AX36">
-        <f t="shared" si="15"/>
-        <v>1800</v>
-      </c>
-      <c r="AY36">
-        <f t="shared" si="15"/>
-        <v>1836</v>
-      </c>
-      <c r="AZ36">
-        <f t="shared" si="15"/>
-        <v>1872</v>
-      </c>
-      <c r="BA36">
-        <f t="shared" si="15"/>
-        <v>1908</v>
-      </c>
-      <c r="BB36">
-        <f t="shared" si="15"/>
-        <v>1944</v>
-      </c>
-      <c r="BC36">
-        <f t="shared" si="15"/>
-        <v>1980</v>
-      </c>
-      <c r="BD36">
-        <f t="shared" si="15"/>
-        <v>2016</v>
-      </c>
+      <c r="AT36" s="114"/>
+      <c r="AU36" s="114"/>
+      <c r="AV36" s="114"/>
+      <c r="AW36" s="114"/>
+      <c r="AX36" s="114"/>
+      <c r="AY36" s="114"/>
+      <c r="AZ36" s="114"/>
+      <c r="BA36" s="114"/>
+      <c r="BB36" s="114"/>
+      <c r="BC36" s="114"/>
+      <c r="BD36" s="114"/>
       <c r="BE36">
         <f t="shared" si="15"/>
         <v>2052</v>
@@ -12971,50 +12651,17 @@
         <f t="shared" si="14"/>
         <v>1665</v>
       </c>
-      <c r="AT37">
-        <f t="shared" si="14"/>
-        <v>1702</v>
-      </c>
-      <c r="AU37">
-        <f t="shared" si="15"/>
-        <v>1739</v>
-      </c>
-      <c r="AV37">
-        <f t="shared" si="15"/>
-        <v>1776</v>
-      </c>
-      <c r="AW37">
-        <f t="shared" si="15"/>
-        <v>1813</v>
-      </c>
-      <c r="AX37">
-        <f t="shared" si="15"/>
-        <v>1850</v>
-      </c>
-      <c r="AY37">
-        <f t="shared" si="15"/>
-        <v>1887</v>
-      </c>
-      <c r="AZ37">
-        <f t="shared" si="15"/>
-        <v>1924</v>
-      </c>
-      <c r="BA37">
-        <f t="shared" si="15"/>
-        <v>1961</v>
-      </c>
-      <c r="BB37">
-        <f t="shared" si="15"/>
-        <v>1998</v>
-      </c>
-      <c r="BC37">
-        <f t="shared" si="15"/>
-        <v>2035</v>
-      </c>
-      <c r="BD37">
-        <f t="shared" si="15"/>
-        <v>2072</v>
-      </c>
+      <c r="AT37" s="114"/>
+      <c r="AU37" s="114"/>
+      <c r="AV37" s="114"/>
+      <c r="AW37" s="114"/>
+      <c r="AX37" s="114"/>
+      <c r="AY37" s="114"/>
+      <c r="AZ37" s="114"/>
+      <c r="BA37" s="114"/>
+      <c r="BB37" s="114"/>
+      <c r="BC37" s="114"/>
+      <c r="BD37" s="114"/>
       <c r="BE37">
         <f t="shared" si="15"/>
         <v>2109</v>
@@ -13289,50 +12936,17 @@
         <f t="shared" si="14"/>
         <v>1710</v>
       </c>
-      <c r="AT38">
-        <f t="shared" si="14"/>
-        <v>1748</v>
-      </c>
-      <c r="AU38">
-        <f t="shared" si="15"/>
-        <v>1786</v>
-      </c>
-      <c r="AV38">
-        <f t="shared" si="15"/>
-        <v>1824</v>
-      </c>
-      <c r="AW38">
-        <f t="shared" si="15"/>
-        <v>1862</v>
-      </c>
-      <c r="AX38">
-        <f t="shared" si="15"/>
-        <v>1900</v>
-      </c>
-      <c r="AY38">
-        <f t="shared" si="15"/>
-        <v>1938</v>
-      </c>
-      <c r="AZ38">
-        <f t="shared" si="15"/>
-        <v>1976</v>
-      </c>
-      <c r="BA38">
-        <f t="shared" si="15"/>
-        <v>2014</v>
-      </c>
-      <c r="BB38">
-        <f t="shared" si="15"/>
-        <v>2052</v>
-      </c>
-      <c r="BC38">
-        <f t="shared" si="15"/>
-        <v>2090</v>
-      </c>
-      <c r="BD38">
-        <f t="shared" si="15"/>
-        <v>2128</v>
-      </c>
+      <c r="AT38" s="114"/>
+      <c r="AU38" s="114"/>
+      <c r="AV38" s="114"/>
+      <c r="AW38" s="114"/>
+      <c r="AX38" s="114"/>
+      <c r="AY38" s="114"/>
+      <c r="AZ38" s="114"/>
+      <c r="BA38" s="114"/>
+      <c r="BB38" s="114"/>
+      <c r="BC38" s="114"/>
+      <c r="BD38" s="114"/>
       <c r="BE38">
         <f t="shared" si="15"/>
         <v>2166</v>
@@ -13440,7 +13054,7 @@
     </row>
     <row r="39" spans="1:82" x14ac:dyDescent="0.25">
       <c r="A39">
-        <f t="shared" ref="A39:P79" si="17">ROW()*COLUMN()</f>
+        <f t="shared" ref="A39:P75" si="17">ROW()*COLUMN()</f>
         <v>39</v>
       </c>
       <c r="B39" s="20">
@@ -13492,7 +13106,7 @@
         <v>624</v>
       </c>
       <c r="Q39">
-        <f t="shared" ref="Q39:AF79" si="18">ROW()*COLUMN()</f>
+        <f t="shared" ref="Q39:AF58" si="18">ROW()*COLUMN()</f>
         <v>663</v>
       </c>
       <c r="R39">
@@ -13607,50 +13221,17 @@
         <f t="shared" si="14"/>
         <v>1755</v>
       </c>
-      <c r="AT39">
-        <f t="shared" si="14"/>
-        <v>1794</v>
-      </c>
-      <c r="AU39">
-        <f t="shared" si="15"/>
-        <v>1833</v>
-      </c>
-      <c r="AV39">
-        <f t="shared" si="15"/>
-        <v>1872</v>
-      </c>
-      <c r="AW39">
-        <f t="shared" si="15"/>
-        <v>1911</v>
-      </c>
-      <c r="AX39">
-        <f t="shared" si="15"/>
-        <v>1950</v>
-      </c>
-      <c r="AY39">
-        <f t="shared" si="15"/>
-        <v>1989</v>
-      </c>
-      <c r="AZ39">
-        <f t="shared" si="15"/>
-        <v>2028</v>
-      </c>
-      <c r="BA39">
-        <f t="shared" si="15"/>
-        <v>2067</v>
-      </c>
-      <c r="BB39">
-        <f t="shared" si="15"/>
-        <v>2106</v>
-      </c>
-      <c r="BC39">
-        <f t="shared" si="15"/>
-        <v>2145</v>
-      </c>
-      <c r="BD39">
-        <f t="shared" si="15"/>
-        <v>2184</v>
-      </c>
+      <c r="AT39" s="114"/>
+      <c r="AU39" s="114"/>
+      <c r="AV39" s="114"/>
+      <c r="AW39" s="114"/>
+      <c r="AX39" s="114"/>
+      <c r="AY39" s="114"/>
+      <c r="AZ39" s="114"/>
+      <c r="BA39" s="114"/>
+      <c r="BB39" s="114"/>
+      <c r="BC39" s="114"/>
+      <c r="BD39" s="114"/>
       <c r="BE39">
         <f t="shared" si="15"/>
         <v>2223</v>
@@ -13925,50 +13506,17 @@
         <f t="shared" si="14"/>
         <v>1800</v>
       </c>
-      <c r="AT40">
-        <f t="shared" si="14"/>
-        <v>1840</v>
-      </c>
-      <c r="AU40">
-        <f t="shared" si="15"/>
-        <v>1880</v>
-      </c>
-      <c r="AV40">
-        <f t="shared" si="15"/>
-        <v>1920</v>
-      </c>
-      <c r="AW40">
-        <f t="shared" si="15"/>
-        <v>1960</v>
-      </c>
-      <c r="AX40">
-        <f t="shared" si="15"/>
-        <v>2000</v>
-      </c>
-      <c r="AY40">
-        <f t="shared" si="15"/>
-        <v>2040</v>
-      </c>
-      <c r="AZ40">
-        <f t="shared" si="15"/>
-        <v>2080</v>
-      </c>
-      <c r="BA40">
-        <f t="shared" si="15"/>
-        <v>2120</v>
-      </c>
-      <c r="BB40">
-        <f t="shared" si="15"/>
-        <v>2160</v>
-      </c>
-      <c r="BC40">
-        <f t="shared" si="15"/>
-        <v>2200</v>
-      </c>
-      <c r="BD40">
-        <f t="shared" si="15"/>
-        <v>2240</v>
-      </c>
+      <c r="AT40" s="114"/>
+      <c r="AU40" s="114"/>
+      <c r="AV40" s="114"/>
+      <c r="AW40" s="114"/>
+      <c r="AX40" s="114"/>
+      <c r="AY40" s="114"/>
+      <c r="AZ40" s="114"/>
+      <c r="BA40" s="114"/>
+      <c r="BB40" s="114"/>
+      <c r="BC40" s="114"/>
+      <c r="BD40" s="114"/>
       <c r="BE40">
         <f t="shared" si="15"/>
         <v>2280</v>
@@ -14243,50 +13791,17 @@
         <f t="shared" si="14"/>
         <v>1845</v>
       </c>
-      <c r="AT41">
-        <f t="shared" si="14"/>
-        <v>1886</v>
-      </c>
-      <c r="AU41">
-        <f t="shared" si="15"/>
-        <v>1927</v>
-      </c>
-      <c r="AV41">
-        <f t="shared" si="15"/>
-        <v>1968</v>
-      </c>
-      <c r="AW41">
-        <f t="shared" si="15"/>
-        <v>2009</v>
-      </c>
-      <c r="AX41">
-        <f t="shared" si="15"/>
-        <v>2050</v>
-      </c>
-      <c r="AY41">
-        <f t="shared" si="15"/>
-        <v>2091</v>
-      </c>
-      <c r="AZ41">
-        <f t="shared" si="15"/>
-        <v>2132</v>
-      </c>
-      <c r="BA41">
-        <f t="shared" si="15"/>
-        <v>2173</v>
-      </c>
-      <c r="BB41">
-        <f t="shared" si="15"/>
-        <v>2214</v>
-      </c>
-      <c r="BC41">
-        <f t="shared" si="15"/>
-        <v>2255</v>
-      </c>
-      <c r="BD41">
-        <f t="shared" si="15"/>
-        <v>2296</v>
-      </c>
+      <c r="AT41" s="114"/>
+      <c r="AU41" s="114"/>
+      <c r="AV41" s="114"/>
+      <c r="AW41" s="114"/>
+      <c r="AX41" s="114"/>
+      <c r="AY41" s="114"/>
+      <c r="AZ41" s="114"/>
+      <c r="BA41" s="114"/>
+      <c r="BB41" s="114"/>
+      <c r="BC41" s="114"/>
+      <c r="BD41" s="114"/>
       <c r="BE41">
         <f t="shared" si="15"/>
         <v>2337</v>
@@ -14561,50 +14076,17 @@
         <f t="shared" si="14"/>
         <v>1890</v>
       </c>
-      <c r="AT42">
-        <f t="shared" si="14"/>
-        <v>1932</v>
-      </c>
-      <c r="AU42">
-        <f t="shared" si="15"/>
-        <v>1974</v>
-      </c>
-      <c r="AV42">
-        <f t="shared" si="15"/>
-        <v>2016</v>
-      </c>
-      <c r="AW42">
-        <f t="shared" si="15"/>
-        <v>2058</v>
-      </c>
-      <c r="AX42">
-        <f t="shared" si="15"/>
-        <v>2100</v>
-      </c>
-      <c r="AY42">
-        <f t="shared" si="15"/>
-        <v>2142</v>
-      </c>
-      <c r="AZ42">
-        <f t="shared" si="15"/>
-        <v>2184</v>
-      </c>
-      <c r="BA42">
-        <f t="shared" si="15"/>
-        <v>2226</v>
-      </c>
-      <c r="BB42">
-        <f t="shared" si="15"/>
-        <v>2268</v>
-      </c>
-      <c r="BC42">
-        <f t="shared" si="15"/>
-        <v>2310</v>
-      </c>
-      <c r="BD42">
-        <f t="shared" si="15"/>
-        <v>2352</v>
-      </c>
+      <c r="AT42" s="114"/>
+      <c r="AU42" s="114"/>
+      <c r="AV42" s="114"/>
+      <c r="AW42" s="114"/>
+      <c r="AX42" s="114"/>
+      <c r="AY42" s="114"/>
+      <c r="AZ42" s="114"/>
+      <c r="BA42" s="114"/>
+      <c r="BB42" s="114"/>
+      <c r="BC42" s="114"/>
+      <c r="BD42" s="114"/>
       <c r="BE42">
         <f t="shared" si="15"/>
         <v>2394</v>
@@ -14879,50 +14361,17 @@
         <f t="shared" si="14"/>
         <v>1935</v>
       </c>
-      <c r="AT43">
-        <f t="shared" si="14"/>
-        <v>1978</v>
-      </c>
-      <c r="AU43">
-        <f t="shared" si="15"/>
-        <v>2021</v>
-      </c>
-      <c r="AV43">
-        <f t="shared" si="15"/>
-        <v>2064</v>
-      </c>
-      <c r="AW43">
-        <f t="shared" si="15"/>
-        <v>2107</v>
-      </c>
-      <c r="AX43">
-        <f t="shared" si="15"/>
-        <v>2150</v>
-      </c>
-      <c r="AY43">
-        <f t="shared" si="15"/>
-        <v>2193</v>
-      </c>
-      <c r="AZ43">
-        <f t="shared" si="15"/>
-        <v>2236</v>
-      </c>
-      <c r="BA43">
-        <f t="shared" si="15"/>
-        <v>2279</v>
-      </c>
-      <c r="BB43">
-        <f t="shared" si="15"/>
-        <v>2322</v>
-      </c>
-      <c r="BC43">
-        <f t="shared" si="15"/>
-        <v>2365</v>
-      </c>
-      <c r="BD43">
-        <f t="shared" si="15"/>
-        <v>2408</v>
-      </c>
+      <c r="AT43" s="114"/>
+      <c r="AU43" s="114"/>
+      <c r="AV43" s="114"/>
+      <c r="AW43" s="114"/>
+      <c r="AX43" s="114"/>
+      <c r="AY43" s="114"/>
+      <c r="AZ43" s="114"/>
+      <c r="BA43" s="114"/>
+      <c r="BB43" s="114"/>
+      <c r="BC43" s="114"/>
+      <c r="BD43" s="114"/>
       <c r="BE43">
         <f t="shared" si="15"/>
         <v>2451</v>
@@ -15197,50 +14646,17 @@
         <f t="shared" si="14"/>
         <v>1980</v>
       </c>
-      <c r="AT44">
-        <f t="shared" si="14"/>
-        <v>2024</v>
-      </c>
-      <c r="AU44">
-        <f t="shared" si="15"/>
-        <v>2068</v>
-      </c>
-      <c r="AV44">
-        <f t="shared" si="15"/>
-        <v>2112</v>
-      </c>
-      <c r="AW44">
-        <f t="shared" si="15"/>
-        <v>2156</v>
-      </c>
-      <c r="AX44">
-        <f t="shared" si="15"/>
-        <v>2200</v>
-      </c>
-      <c r="AY44">
-        <f t="shared" si="15"/>
-        <v>2244</v>
-      </c>
-      <c r="AZ44">
-        <f t="shared" si="15"/>
-        <v>2288</v>
-      </c>
-      <c r="BA44">
-        <f t="shared" si="15"/>
-        <v>2332</v>
-      </c>
-      <c r="BB44">
-        <f t="shared" si="15"/>
-        <v>2376</v>
-      </c>
-      <c r="BC44">
-        <f t="shared" si="15"/>
-        <v>2420</v>
-      </c>
-      <c r="BD44">
-        <f t="shared" si="15"/>
-        <v>2464</v>
-      </c>
+      <c r="AT44" s="114"/>
+      <c r="AU44" s="114"/>
+      <c r="AV44" s="114"/>
+      <c r="AW44" s="114"/>
+      <c r="AX44" s="114"/>
+      <c r="AY44" s="114"/>
+      <c r="AZ44" s="114"/>
+      <c r="BA44" s="114"/>
+      <c r="BB44" s="114"/>
+      <c r="BC44" s="114"/>
+      <c r="BD44" s="114"/>
       <c r="BE44">
         <f t="shared" si="15"/>
         <v>2508</v>
@@ -15515,50 +14931,17 @@
         <f t="shared" si="14"/>
         <v>2025</v>
       </c>
-      <c r="AT45">
-        <f t="shared" si="14"/>
-        <v>2070</v>
-      </c>
-      <c r="AU45">
-        <f t="shared" si="15"/>
-        <v>2115</v>
-      </c>
-      <c r="AV45">
-        <f t="shared" si="15"/>
-        <v>2160</v>
-      </c>
-      <c r="AW45">
-        <f t="shared" si="15"/>
-        <v>2205</v>
-      </c>
-      <c r="AX45">
-        <f t="shared" si="15"/>
-        <v>2250</v>
-      </c>
-      <c r="AY45">
-        <f t="shared" si="15"/>
-        <v>2295</v>
-      </c>
-      <c r="AZ45">
-        <f t="shared" si="15"/>
-        <v>2340</v>
-      </c>
-      <c r="BA45">
-        <f t="shared" si="15"/>
-        <v>2385</v>
-      </c>
-      <c r="BB45">
-        <f t="shared" si="15"/>
-        <v>2430</v>
-      </c>
-      <c r="BC45">
-        <f t="shared" si="15"/>
-        <v>2475</v>
-      </c>
-      <c r="BD45">
-        <f t="shared" si="15"/>
-        <v>2520</v>
-      </c>
+      <c r="AT45" s="114"/>
+      <c r="AU45" s="114"/>
+      <c r="AV45" s="114"/>
+      <c r="AW45" s="114"/>
+      <c r="AX45" s="114"/>
+      <c r="AY45" s="114"/>
+      <c r="AZ45" s="114"/>
+      <c r="BA45" s="114"/>
+      <c r="BB45" s="114"/>
+      <c r="BC45" s="114"/>
+      <c r="BD45" s="114"/>
       <c r="BE45">
         <f t="shared" si="15"/>
         <v>2565</v>
@@ -15833,50 +15216,17 @@
         <f t="shared" si="14"/>
         <v>2070</v>
       </c>
-      <c r="AT46">
-        <f t="shared" si="14"/>
-        <v>2116</v>
-      </c>
-      <c r="AU46">
-        <f t="shared" si="15"/>
-        <v>2162</v>
-      </c>
-      <c r="AV46">
-        <f t="shared" si="15"/>
-        <v>2208</v>
-      </c>
-      <c r="AW46">
-        <f t="shared" si="15"/>
-        <v>2254</v>
-      </c>
-      <c r="AX46">
-        <f t="shared" si="15"/>
-        <v>2300</v>
-      </c>
-      <c r="AY46">
-        <f t="shared" si="15"/>
-        <v>2346</v>
-      </c>
-      <c r="AZ46">
-        <f t="shared" si="15"/>
-        <v>2392</v>
-      </c>
-      <c r="BA46">
-        <f t="shared" si="15"/>
-        <v>2438</v>
-      </c>
-      <c r="BB46">
-        <f t="shared" si="15"/>
-        <v>2484</v>
-      </c>
-      <c r="BC46">
-        <f t="shared" si="15"/>
-        <v>2530</v>
-      </c>
-      <c r="BD46">
-        <f t="shared" si="15"/>
-        <v>2576</v>
-      </c>
+      <c r="AT46" s="114"/>
+      <c r="AU46" s="114"/>
+      <c r="AV46" s="114"/>
+      <c r="AW46" s="114"/>
+      <c r="AX46" s="114"/>
+      <c r="AY46" s="114"/>
+      <c r="AZ46" s="114"/>
+      <c r="BA46" s="114"/>
+      <c r="BB46" s="114"/>
+      <c r="BC46" s="114"/>
+      <c r="BD46" s="114"/>
       <c r="BE46">
         <f t="shared" si="15"/>
         <v>2622</v>
@@ -16100,7 +15450,7 @@
         <v>1504</v>
       </c>
       <c r="AG47">
-        <f t="shared" ref="AG47:AT79" si="19">ROW()*COLUMN()</f>
+        <f t="shared" ref="AG47:AT67" si="19">ROW()*COLUMN()</f>
         <v>1551</v>
       </c>
       <c r="AH47">
@@ -16151,50 +15501,17 @@
         <f t="shared" si="19"/>
         <v>2115</v>
       </c>
-      <c r="AT47">
-        <f t="shared" si="19"/>
-        <v>2162</v>
-      </c>
-      <c r="AU47">
-        <f t="shared" si="15"/>
-        <v>2209</v>
-      </c>
-      <c r="AV47">
-        <f t="shared" si="15"/>
-        <v>2256</v>
-      </c>
-      <c r="AW47">
-        <f t="shared" si="15"/>
-        <v>2303</v>
-      </c>
-      <c r="AX47">
-        <f t="shared" si="15"/>
-        <v>2350</v>
-      </c>
-      <c r="AY47">
-        <f t="shared" si="15"/>
-        <v>2397</v>
-      </c>
-      <c r="AZ47">
-        <f t="shared" si="15"/>
-        <v>2444</v>
-      </c>
-      <c r="BA47">
-        <f t="shared" si="15"/>
-        <v>2491</v>
-      </c>
-      <c r="BB47">
-        <f t="shared" si="15"/>
-        <v>2538</v>
-      </c>
-      <c r="BC47">
-        <f t="shared" si="15"/>
-        <v>2585</v>
-      </c>
-      <c r="BD47">
-        <f t="shared" si="15"/>
-        <v>2632</v>
-      </c>
+      <c r="AT47" s="114"/>
+      <c r="AU47" s="114"/>
+      <c r="AV47" s="114"/>
+      <c r="AW47" s="114"/>
+      <c r="AX47" s="114"/>
+      <c r="AY47" s="114"/>
+      <c r="AZ47" s="114"/>
+      <c r="BA47" s="114"/>
+      <c r="BB47" s="114"/>
+      <c r="BC47" s="114"/>
+      <c r="BD47" s="114"/>
       <c r="BE47">
         <f t="shared" si="15"/>
         <v>2679</v>
@@ -16469,50 +15786,17 @@
         <f t="shared" si="19"/>
         <v>2160</v>
       </c>
-      <c r="AT48">
-        <f t="shared" si="19"/>
-        <v>2208</v>
-      </c>
-      <c r="AU48">
-        <f t="shared" si="15"/>
-        <v>2256</v>
-      </c>
-      <c r="AV48">
-        <f t="shared" si="15"/>
-        <v>2304</v>
-      </c>
-      <c r="AW48">
-        <f t="shared" si="15"/>
-        <v>2352</v>
-      </c>
-      <c r="AX48">
-        <f t="shared" si="15"/>
-        <v>2400</v>
-      </c>
-      <c r="AY48">
-        <f t="shared" si="15"/>
-        <v>2448</v>
-      </c>
-      <c r="AZ48">
-        <f t="shared" si="15"/>
-        <v>2496</v>
-      </c>
-      <c r="BA48">
-        <f t="shared" si="15"/>
-        <v>2544</v>
-      </c>
-      <c r="BB48">
-        <f t="shared" si="15"/>
-        <v>2592</v>
-      </c>
-      <c r="BC48">
-        <f t="shared" si="15"/>
-        <v>2640</v>
-      </c>
-      <c r="BD48">
-        <f t="shared" si="15"/>
-        <v>2688</v>
-      </c>
+      <c r="AT48" s="114"/>
+      <c r="AU48" s="114"/>
+      <c r="AV48" s="114"/>
+      <c r="AW48" s="114"/>
+      <c r="AX48" s="114"/>
+      <c r="AY48" s="114"/>
+      <c r="AZ48" s="114"/>
+      <c r="BA48" s="114"/>
+      <c r="BB48" s="114"/>
+      <c r="BC48" s="114"/>
+      <c r="BD48" s="114"/>
       <c r="BE48">
         <f t="shared" si="15"/>
         <v>2736</v>
@@ -16787,50 +16071,17 @@
         <f t="shared" si="19"/>
         <v>2205</v>
       </c>
-      <c r="AT49">
-        <f t="shared" si="19"/>
-        <v>2254</v>
-      </c>
-      <c r="AU49">
-        <f t="shared" si="15"/>
-        <v>2303</v>
-      </c>
-      <c r="AV49">
-        <f t="shared" si="15"/>
-        <v>2352</v>
-      </c>
-      <c r="AW49">
-        <f t="shared" si="15"/>
-        <v>2401</v>
-      </c>
-      <c r="AX49">
-        <f t="shared" si="15"/>
-        <v>2450</v>
-      </c>
-      <c r="AY49">
-        <f t="shared" si="15"/>
-        <v>2499</v>
-      </c>
-      <c r="AZ49">
-        <f t="shared" si="15"/>
-        <v>2548</v>
-      </c>
-      <c r="BA49">
-        <f t="shared" si="15"/>
-        <v>2597</v>
-      </c>
-      <c r="BB49">
-        <f t="shared" si="15"/>
-        <v>2646</v>
-      </c>
-      <c r="BC49">
-        <f t="shared" si="15"/>
-        <v>2695</v>
-      </c>
-      <c r="BD49">
-        <f t="shared" si="15"/>
-        <v>2744</v>
-      </c>
+      <c r="AT49" s="114"/>
+      <c r="AU49" s="114"/>
+      <c r="AV49" s="114"/>
+      <c r="AW49" s="114"/>
+      <c r="AX49" s="114"/>
+      <c r="AY49" s="114"/>
+      <c r="AZ49" s="114"/>
+      <c r="BA49" s="114"/>
+      <c r="BB49" s="114"/>
+      <c r="BC49" s="114"/>
+      <c r="BD49" s="114"/>
       <c r="BE49">
         <f t="shared" si="15"/>
         <v>2793</v>
@@ -17105,50 +16356,17 @@
         <f t="shared" si="19"/>
         <v>2250</v>
       </c>
-      <c r="AT50">
-        <f t="shared" si="19"/>
-        <v>2300</v>
-      </c>
-      <c r="AU50">
-        <f t="shared" si="15"/>
-        <v>2350</v>
-      </c>
-      <c r="AV50">
-        <f t="shared" si="15"/>
-        <v>2400</v>
-      </c>
-      <c r="AW50">
-        <f t="shared" si="15"/>
-        <v>2450</v>
-      </c>
-      <c r="AX50">
-        <f t="shared" si="15"/>
-        <v>2500</v>
-      </c>
-      <c r="AY50">
-        <f t="shared" si="15"/>
-        <v>2550</v>
-      </c>
-      <c r="AZ50">
-        <f t="shared" si="15"/>
-        <v>2600</v>
-      </c>
-      <c r="BA50">
-        <f t="shared" si="15"/>
-        <v>2650</v>
-      </c>
-      <c r="BB50">
-        <f t="shared" si="15"/>
-        <v>2700</v>
-      </c>
-      <c r="BC50">
-        <f t="shared" si="15"/>
-        <v>2750</v>
-      </c>
-      <c r="BD50">
-        <f t="shared" si="15"/>
-        <v>2800</v>
-      </c>
+      <c r="AT50" s="114"/>
+      <c r="AU50" s="114"/>
+      <c r="AV50" s="114"/>
+      <c r="AW50" s="114"/>
+      <c r="AX50" s="114"/>
+      <c r="AY50" s="114"/>
+      <c r="AZ50" s="114"/>
+      <c r="BA50" s="114"/>
+      <c r="BB50" s="114"/>
+      <c r="BC50" s="114"/>
+      <c r="BD50" s="114"/>
       <c r="BE50">
         <f t="shared" si="15"/>
         <v>2850</v>
@@ -17423,50 +16641,17 @@
         <f t="shared" si="19"/>
         <v>2295</v>
       </c>
-      <c r="AT51">
-        <f t="shared" si="19"/>
-        <v>2346</v>
-      </c>
-      <c r="AU51">
-        <f t="shared" si="15"/>
-        <v>2397</v>
-      </c>
-      <c r="AV51">
-        <f t="shared" si="15"/>
-        <v>2448</v>
-      </c>
-      <c r="AW51">
-        <f t="shared" si="15"/>
-        <v>2499</v>
-      </c>
-      <c r="AX51">
-        <f t="shared" si="15"/>
-        <v>2550</v>
-      </c>
-      <c r="AY51">
-        <f t="shared" si="15"/>
-        <v>2601</v>
-      </c>
-      <c r="AZ51">
-        <f t="shared" si="15"/>
-        <v>2652</v>
-      </c>
-      <c r="BA51">
-        <f t="shared" si="15"/>
-        <v>2703</v>
-      </c>
-      <c r="BB51">
-        <f t="shared" si="15"/>
-        <v>2754</v>
-      </c>
-      <c r="BC51">
-        <f t="shared" si="15"/>
-        <v>2805</v>
-      </c>
-      <c r="BD51">
-        <f t="shared" si="15"/>
-        <v>2856</v>
-      </c>
+      <c r="AT51" s="114"/>
+      <c r="AU51" s="114"/>
+      <c r="AV51" s="114"/>
+      <c r="AW51" s="114"/>
+      <c r="AX51" s="114"/>
+      <c r="AY51" s="114"/>
+      <c r="AZ51" s="114"/>
+      <c r="BA51" s="114"/>
+      <c r="BB51" s="114"/>
+      <c r="BC51" s="114"/>
+      <c r="BD51" s="114"/>
       <c r="BE51">
         <f t="shared" si="15"/>
         <v>2907</v>
@@ -17480,7 +16665,7 @@
         <v>3009</v>
       </c>
       <c r="BH51">
-        <f t="shared" ref="AU51:BH79" si="21">ROW()*COLUMN()</f>
+        <f t="shared" ref="AU51:BH70" si="21">ROW()*COLUMN()</f>
         <v>3060</v>
       </c>
       <c r="BI51">
@@ -19852,7 +19037,7 @@
         <v>944</v>
       </c>
       <c r="Q59">
-        <f t="shared" ref="Q59:X79" si="23">ROW()*COLUMN()</f>
+        <f t="shared" ref="Q59:X74" si="23">ROW()*COLUMN()</f>
         <v>1003</v>
       </c>
       <c r="R59">
@@ -26477,7 +25662,13 @@
       </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
+  <mergeCells count="11">
+    <mergeCell ref="AT28:BD51"/>
+    <mergeCell ref="E6:F8"/>
+    <mergeCell ref="E10:F12"/>
+    <mergeCell ref="E14:F16"/>
+    <mergeCell ref="E2:F3"/>
+    <mergeCell ref="R2:S3"/>
     <mergeCell ref="K16:X16"/>
     <mergeCell ref="K22:N24"/>
     <mergeCell ref="S22:X24"/>

</xml_diff>